<commit_message>
Corrected tech name in template.
</commit_message>
<xml_diff>
--- a/backend/fms_core/static/submission_templates/Library_conversion_v4_4_0.xlsx
+++ b/backend/fms_core/static/submission_templates/Library_conversion_v4_4_0.xlsx
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="150" uniqueCount="103">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="152" uniqueCount="105">
   <si>
     <t xml:space="preserve">Library Conversion Template</t>
   </si>
@@ -331,7 +331,7 @@
     <t xml:space="preserve">Step complete - Move to next step</t>
   </si>
   <si>
-    <t xml:space="preserve">Elizabeth Caron</t>
+    <t xml:space="preserve">Patrick Willett</t>
   </si>
   <si>
     <t xml:space="preserve">MGI_Conversion_AppB</t>
@@ -346,7 +346,7 @@
     <t xml:space="preserve">Sample failed - Remove sample from study workflow</t>
   </si>
   <si>
-    <t xml:space="preserve">Patrick Willett</t>
+    <t xml:space="preserve">Ariane Boisclair</t>
   </si>
   <si>
     <t xml:space="preserve">MGI_Conversion_AppC</t>
@@ -361,7 +361,7 @@
     <t xml:space="preserve">Repeat step - Move to next step and repeat current step</t>
   </si>
   <si>
-    <t xml:space="preserve">Ariane Boisclair</t>
+    <t xml:space="preserve">Marlon Amersi</t>
   </si>
   <si>
     <t xml:space="preserve">Eppendorf 4 Pre-PCR</t>
@@ -373,7 +373,7 @@
     <t xml:space="preserve">Ignore workflow - Do not register as part of a workflow</t>
   </si>
   <si>
-    <t xml:space="preserve">Marlon Amersi</t>
+    <t xml:space="preserve">Antoine Farley</t>
   </si>
   <si>
     <t xml:space="preserve">Biometra Rouge</t>
@@ -382,7 +382,7 @@
     <t xml:space="preserve">Tube Strip 3x1</t>
   </si>
   <si>
-    <t xml:space="preserve">Antoine Farley</t>
+    <t xml:space="preserve">Lena Li</t>
   </si>
   <si>
     <t xml:space="preserve">Eppendorf 1 Post-PCR</t>
@@ -391,7 +391,7 @@
     <t xml:space="preserve">Tube Strip 4x1</t>
   </si>
   <si>
-    <t xml:space="preserve">Lena Li</t>
+    <t xml:space="preserve">Girija Daliah</t>
   </si>
   <si>
     <t xml:space="preserve">Eppendorf 2 Post-PCR</t>
@@ -400,19 +400,25 @@
     <t xml:space="preserve">Tube Strip 5x1</t>
   </si>
   <si>
-    <t xml:space="preserve">Girija Daliah</t>
+    <t xml:space="preserve">Marie-Michelle Simon</t>
   </si>
   <si>
     <t xml:space="preserve">Tube Strip 6x1</t>
   </si>
   <si>
-    <t xml:space="preserve">Marie-Michelle Simons</t>
+    <t xml:space="preserve">Nadège Zaghdoudi Allan</t>
   </si>
   <si>
     <t xml:space="preserve">Tube Strip 7x1</t>
   </si>
   <si>
+    <t xml:space="preserve">Daniel Vincent</t>
+  </si>
+  <si>
     <t xml:space="preserve">Tube Strip 8x1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Esen Sokullu</t>
   </si>
 </sst>
 </file>
@@ -632,7 +638,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="37">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -777,6 +783,10 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -855,7 +865,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AC1048576"/>
-  <sheetFormatPr defaultColWidth="11.27734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.28125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="32.11"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="2" style="0" width="24.78"/>
@@ -8715,26 +8725,26 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="4">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C7:C380" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="C7:C380" type="list">
       <formula1>Index!$A$2</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F7:F383" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="F7:F383" type="list">
       <formula1>Index!$C$2:$C$4</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H380" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H7:H380" type="list">
       <formula1>Index!$D$2:$D$8</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E7:E380" type="list">
-      <formula1>Index!$B$2:$B$10</formula1>
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="E7:E380" type="list">
+      <formula1>Index!$B$2:$B$12</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -8748,7 +8758,7 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:AB1048576"/>
-  <sheetFormatPr defaultColWidth="11.27734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.28125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="1" style="0" width="24.33"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="34.67"/>
@@ -21920,22 +21930,22 @@
     <row r="1048576" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H5:H480" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="H5:H480" type="list">
       <formula1>Index!$E$2:$E$11</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A5:A381" type="list">
+    <dataValidation allowBlank="true" operator="between" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="A5:A381" type="list">
       <formula1>'Conversion Batch'!$A$7:$A$380</formula1>
       <formula2>0</formula2>
     </dataValidation>
-    <dataValidation allowBlank="true" errorStyle="stop" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R5:R381" type="list">
+    <dataValidation allowBlank="true" operator="equal" showDropDown="false" showErrorMessage="true" showInputMessage="false" sqref="R5:R381" type="list">
       <formula1>Index!$F$2:$F$5</formula1>
       <formula2>0</formula2>
     </dataValidation>
   </dataValidations>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>
@@ -22290,7 +22300,7 @@
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"Page &amp;P</oddFooter>
@@ -22304,10 +22314,10 @@
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
   <dimension ref="A1:J1000"/>
-  <sheetFormatPr defaultColWidth="11.27734375" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <sheetFormatPr defaultColWidth="11.28125" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="17.78"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="18.78"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="22.79"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="22.44"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="0" width="32"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="0" width="15.79"/>
@@ -22343,7 +22353,7 @@
       <c r="A2" s="15" t="s">
         <v>69</v>
       </c>
-      <c r="B2" s="15" t="s">
+      <c r="B2" s="36" t="s">
         <v>70</v>
       </c>
       <c r="C2" s="13" t="s">
@@ -22360,7 +22370,7 @@
       </c>
     </row>
     <row r="3" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B3" s="15" t="s">
+      <c r="B3" s="36" t="s">
         <v>75</v>
       </c>
       <c r="C3" s="13" t="s">
@@ -22378,7 +22388,7 @@
       <c r="J3" s="13"/>
     </row>
     <row r="4" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B4" s="15" t="s">
+      <c r="B4" s="36" t="s">
         <v>80</v>
       </c>
       <c r="C4" s="13" t="s">
@@ -22396,7 +22406,7 @@
       <c r="J4" s="13"/>
     </row>
     <row r="5" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B5" s="15" t="s">
+      <c r="B5" s="36" t="s">
         <v>85</v>
       </c>
       <c r="C5" s="13"/>
@@ -22412,7 +22422,7 @@
       <c r="J5" s="13"/>
     </row>
     <row r="6" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B6" s="15" t="s">
+      <c r="B6" s="36" t="s">
         <v>89</v>
       </c>
       <c r="C6" s="13"/>
@@ -22426,7 +22436,7 @@
       <c r="J6" s="13"/>
     </row>
     <row r="7" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B7" s="15" t="s">
+      <c r="B7" s="36" t="s">
         <v>92</v>
       </c>
       <c r="C7" s="13"/>
@@ -22439,7 +22449,7 @@
       <c r="F7" s="13"/>
     </row>
     <row r="8" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B8" s="15" t="s">
+      <c r="B8" s="36" t="s">
         <v>95</v>
       </c>
       <c r="C8" s="13"/>
@@ -22452,7 +22462,7 @@
       <c r="F8" s="13"/>
     </row>
     <row r="9" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B9" s="0" t="s">
+      <c r="B9" s="36" t="s">
         <v>98</v>
       </c>
       <c r="C9" s="13"/>
@@ -22463,7 +22473,7 @@
       <c r="F9" s="13"/>
     </row>
     <row r="10" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B10" s="13" t="s">
+      <c r="B10" s="36" t="s">
         <v>100</v>
       </c>
       <c r="C10" s="13"/>
@@ -22474,16 +22484,20 @@
       <c r="F10" s="13"/>
     </row>
     <row r="11" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B11" s="13"/>
+      <c r="B11" s="36" t="s">
+        <v>102</v>
+      </c>
       <c r="C11" s="13"/>
       <c r="D11" s="15"/>
       <c r="E11" s="15" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="F11" s="13"/>
     </row>
     <row r="12" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B12" s="13"/>
+      <c r="B12" s="36" t="s">
+        <v>104</v>
+      </c>
       <c r="C12" s="13"/>
       <c r="D12" s="13"/>
       <c r="E12" s="13"/>
@@ -23946,6 +23960,7 @@
       <c r="F220" s="13"/>
     </row>
     <row r="221" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B221" s="13"/>
       <c r="F221" s="13"/>
     </row>
     <row r="222" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
@@ -24729,8 +24744,8 @@
     <row r="1000" customFormat="false" ht="15.75" hidden="false" customHeight="true" outlineLevel="0" collapsed="false"/>
   </sheetData>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
-  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511811023622047" footer="0.511811023622047"/>
-  <pageSetup paperSize="1" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.511805555555555" footer="0.511805555555555"/>
+  <pageSetup paperSize="1" scale="100" firstPageNumber="0" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" useFirstPageNumber="false" horizontalDpi="300" verticalDpi="300" copies="1"/>
   <headerFooter differentFirst="false" differentOddEven="false">
     <oddHeader/>
     <oddFooter/>

</xml_diff>